<commit_message>
v4.1: scenario assumptions from Excel sheet; model manual
- input/Database_Rupiah_Bulanan.xlsx: new sheet scenario_inputs, one row
  per scenario x month (h = 1..6): dxy_pct (cumulative DXY vs anchor, %),
  tb_shift_usdbn and flows_shift_idrtn (shift vs Baseline BVARX median;
  blank = month not conditioned). Defaults reproduce the v4 assumptions.
- 06_final_scenarios.do reads and validates the sheet, saves the inputs
  used to T0_scenario_inputs and passes them to Mata.
- 02_bvarx_functions.do: bv_future accepts a monthly DXY path;
  bv_scen_cond and bv_final_run take the per-month inputs.
- 00_master.do: shock globals replaced by global scen_sheet.
- Month labels in scenario tables and charts (06, 10) follow the anchor.
- output/Manual_Model_Simulasi_Rupiah.docx/.pdf: model manual (72 pages)
  with variable inventory, concepts, BMA, BVARX, scenarios, evaluation,
  full results, operations, and references.
- README and CHANGELOG updated; rupiah_bvarx_all.do regenerated.
</commit_message>
<xml_diff>
--- a/input/Database_Rupiah_Bulanan.xlsx
+++ b/input/Database_Rupiah_Bulanan.xlsx
@@ -5,18 +5,19 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO05\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO05\github\Simulasi-Rupiah\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_05E3C132F4969384332F9AE7CB06A3D0D0728861" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDBC71C7-F86A-453A-96DD-B9521C7BD1B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2573" yWindow="2573" windowWidth="16199" windowHeight="9307" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="database_monthly" sheetId="1" r:id="rId1"/>
     <sheet name="flow_components" sheetId="2" r:id="rId2"/>
     <sheet name="rating_events" sheetId="3" r:id="rId3"/>
     <sheet name="sources" sheetId="4" r:id="rId4"/>
+    <sheet name="scenario_inputs" sheetId="7" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="726" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="773" uniqueCount="228">
   <si>
     <t>year</t>
   </si>
@@ -639,17 +640,100 @@
   </si>
   <si>
     <t>Data merupakan latest available vintage, bukan arsip vintage real-time. Untuk backtest, gunakan keterlambatan rilis dan perlakuan revisi yang tepat. Oktober 2026 dikeluarkan karena belum merupakan bulan penuh dan file pasar berhenti 21 Oktober 2026.</t>
+  </si>
+  <si>
+    <t>scenario</t>
+  </si>
+  <si>
+    <t>h</t>
+  </si>
+  <si>
+    <t>dxy_pct</t>
+  </si>
+  <si>
+    <t>tb_shift_usdbn</t>
+  </si>
+  <si>
+    <t>flows_shift_idrtn</t>
+  </si>
+  <si>
+    <t>bulan (info)</t>
+  </si>
+  <si>
+    <t>Baseline</t>
+  </si>
+  <si>
+    <t>Adverse</t>
+  </si>
+  <si>
+    <t>Upside</t>
+  </si>
+  <si>
+    <t>Severe Adverse</t>
+  </si>
+  <si>
+    <t>PETUNJUK (tidak dibaca kode)</t>
+  </si>
+  <si>
+    <t>Anchor (info saja)</t>
+  </si>
+  <si>
+    <t>Dipakai oleh script/06_final_scenarios.do (BVARX), lalu 10_hybrid.do menggeser baseline BMA dengan efek skenario.</t>
+  </si>
+  <si>
+    <t>Sel kuning = input. Abu-abu = diabaikan. Ubah angka saja; jangan ganti nama kolom, nama skenario, atau urutan kolom A-E.</t>
+  </si>
+  <si>
+    <t>scenario: Baseline, Adverse, Upside, Severe Adverse (tetap empat, nama persis seperti ini).</t>
+  </si>
+  <si>
+    <t>h: bulan ke-h setelah anchor (1 = bulan pertama forecast). Harus lengkap 1 sampai H_final (6) untuk tiap skenario.</t>
+  </si>
+  <si>
+    <t>dxy_pct: DXY kumulatif terhadap DXY bulan anchor, dalam persen (2 = DXY 2% lebih tinggi). Wajib diisi semua bulan.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Baseline biasanya 0 (DXY datar). Efek skenario dihitung relatif terhadap Baseline, jadi DXY Baseline ikut menjadi acuan.</t>
+  </si>
+  <si>
+    <t>tb_shift_usdbn: trade balance bulan itu dikunci = median Baseline BVARX + angka ini (USD miliar). Kosong = tidak dikunci.</t>
+  </si>
+  <si>
+    <t>flows_shift_idrtn: net flows asing bulan itu dikunci = median Baseline BVARX + angka ini (Rp triliun). Kosong = tidak dikunci.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Bulan yang tidak dikunci mengikuti dinamika model. Kolom TB dan flows pada baris Baseline diabaikan.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Tanda: negatif = lebih buruk bagi rupiah (TB lebih kecil, arus modal keluar).</t>
+  </si>
+  <si>
+    <t>bulan (info): label bulan dari anchor di sel I3; hanya tampilan, kode memakai anchor dari data.</t>
+  </si>
+  <si>
+    <t>Default (v4): Adverse DXY +2%, TB -1, flows -10; Upside kebalikannya; Severe Adverse DXY +5%, TB -2, flows -30.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   DXY bergerak geometrik menuju angka akhir di h = 6; TB dan flows dikunci di h = 3 dan h = 6.</t>
+  </si>
+  <si>
+    <t>Setelah mengubah: simpan dan tutup file ini, lalu jalankan do "script/00_master.do".</t>
+  </si>
+  <si>
+    <t>Input yang benar-benar dipakai tercatat di output/tables/T0_scenario_inputs.csv.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.000000"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="166" formatCode="0.00"/>
+    <numFmt numFmtId="167" formatCode="0.0"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -663,16 +747,51 @@
       <sz val="10"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9D9D9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEDEDED"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -680,11 +799,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFA6A6A6"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -707,6 +835,28 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="166" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="17" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="17" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="17" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -15110,7 +15260,7 @@
         <v>5</v>
       </c>
       <c r="C162" s="3">
-        <f t="shared" ref="C162:C193" si="30">12*(A162-1960)+B162-1</f>
+        <f t="shared" ref="C162:C166" si="30">12*(A162-1960)+B162-1</f>
         <v>796</v>
       </c>
       <c r="D162" s="4">
@@ -15146,11 +15296,11 @@
         <v>3.75</v>
       </c>
       <c r="N162" s="5">
-        <f t="shared" ref="N162:N193" si="31">(L162+M162)/2</f>
+        <f t="shared" ref="N162:N166" si="31">(L162+M162)/2</f>
         <v>3.625</v>
       </c>
       <c r="O162" s="5">
-        <f t="shared" ref="O162:O193" si="32">K162-N162</f>
+        <f t="shared" ref="O162:O166" si="32">K162-N162</f>
         <v>1.625</v>
       </c>
       <c r="P162" s="3">
@@ -15182,7 +15332,7 @@
         <v>1</v>
       </c>
       <c r="X162" s="3">
-        <f t="shared" ref="X162:X193" si="33">IF(AND(A162&gt;=2014,Y162=1),1,0)</f>
+        <f t="shared" ref="X162:X166" si="33">IF(AND(A162&gt;=2014,Y162=1),1,0)</f>
         <v>1</v>
       </c>
       <c r="Y162" s="3">
@@ -21163,4 +21313,532 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4DB5EDB-214F-45DE-A5D2-A0FA51BCBB70}">
+  <dimension ref="A1:I25"/>
+  <sheetFormatPr defaultRowHeight="12.75"/>
+  <cols>
+    <col min="1" max="1" width="16.5625" style="8" customWidth="1"/>
+    <col min="2" max="2" width="5.5625" style="8" customWidth="1"/>
+    <col min="3" max="3" width="10.5625" style="8" customWidth="1"/>
+    <col min="4" max="4" width="15.5625" style="8" customWidth="1"/>
+    <col min="5" max="5" width="17.5625" style="8" customWidth="1"/>
+    <col min="6" max="6" width="12.5625" style="8" customWidth="1"/>
+    <col min="7" max="7" width="3.5625" style="8" customWidth="1"/>
+    <col min="8" max="8" width="18.5625" style="8" customWidth="1"/>
+    <col min="9" max="16384" width="9" style="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="13.15">
+      <c r="A1" s="10" t="s">
+        <v>201</v>
+      </c>
+      <c r="B1" s="15" t="s">
+        <v>202</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>203</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>204</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>205</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>206</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="13.15">
+      <c r="A2" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="B2" s="16">
+        <v>1</v>
+      </c>
+      <c r="C2" s="11">
+        <v>0</v>
+      </c>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="14">
+        <f>IF($I$3="","",EDATE($I$3,B2))</f>
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="13.15">
+      <c r="A3" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="B3" s="16">
+        <v>2</v>
+      </c>
+      <c r="C3" s="11">
+        <v>0</v>
+      </c>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="14">
+        <f>IF($I$3="","",EDATE($I$3,B3))</f>
+        <v>46327</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>212</v>
+      </c>
+      <c r="I3" s="23">
+        <f>DATE(2026,9,1)</f>
+        <v>46266</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="13.15">
+      <c r="A4" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="B4" s="16">
+        <v>3</v>
+      </c>
+      <c r="C4" s="11">
+        <v>0</v>
+      </c>
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="14">
+        <f>IF($I$3="","",EDATE($I$3,B4))</f>
+        <v>46357</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="13.15">
+      <c r="A5" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="B5" s="16">
+        <v>4</v>
+      </c>
+      <c r="C5" s="11">
+        <v>0</v>
+      </c>
+      <c r="D5" s="12"/>
+      <c r="E5" s="12"/>
+      <c r="F5" s="14">
+        <f>IF($I$3="","",EDATE($I$3,B5))</f>
+        <v>46388</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="13.15">
+      <c r="A6" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="B6" s="16">
+        <v>5</v>
+      </c>
+      <c r="C6" s="11">
+        <v>0</v>
+      </c>
+      <c r="D6" s="12"/>
+      <c r="E6" s="12"/>
+      <c r="F6" s="14">
+        <f>IF($I$3="","",EDATE($I$3,B6))</f>
+        <v>46419</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="13.15">
+      <c r="A7" s="17" t="s">
+        <v>207</v>
+      </c>
+      <c r="B7" s="18">
+        <v>6</v>
+      </c>
+      <c r="C7" s="19">
+        <v>0</v>
+      </c>
+      <c r="D7" s="20"/>
+      <c r="E7" s="20"/>
+      <c r="F7" s="21">
+        <f>IF($I$3="","",EDATE($I$3,B7))</f>
+        <v>46447</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="13.15">
+      <c r="A8" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="B8" s="16">
+        <v>1</v>
+      </c>
+      <c r="C8" s="11">
+        <v>0.33058900000000002</v>
+      </c>
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="14">
+        <f>IF($I$3="","",EDATE($I$3,B8))</f>
+        <v>46296</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="13.15">
+      <c r="A9" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="B9" s="16">
+        <v>2</v>
+      </c>
+      <c r="C9" s="11">
+        <v>0.66227100000000005</v>
+      </c>
+      <c r="D9" s="13"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="14">
+        <f>IF($I$3="","",EDATE($I$3,B9))</f>
+        <v>46327</v>
+      </c>
+      <c r="H9" s="8" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="13.15">
+      <c r="A10" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="B10" s="16">
+        <v>3</v>
+      </c>
+      <c r="C10" s="11">
+        <v>0.99504899999999996</v>
+      </c>
+      <c r="D10" s="13">
+        <v>-1</v>
+      </c>
+      <c r="E10" s="13">
+        <v>-10</v>
+      </c>
+      <c r="F10" s="14">
+        <f>IF($I$3="","",EDATE($I$3,B10))</f>
+        <v>46357</v>
+      </c>
+      <c r="H10" s="8" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="13.15">
+      <c r="A11" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="B11" s="16">
+        <v>4</v>
+      </c>
+      <c r="C11" s="11">
+        <v>1.3289280000000001</v>
+      </c>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="14">
+        <f>IF($I$3="","",EDATE($I$3,B11))</f>
+        <v>46388</v>
+      </c>
+      <c r="H11" s="8" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="13.15">
+      <c r="A12" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="B12" s="16">
+        <v>5</v>
+      </c>
+      <c r="C12" s="11">
+        <v>1.66391</v>
+      </c>
+      <c r="D12" s="13"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="14">
+        <f>IF($I$3="","",EDATE($I$3,B12))</f>
+        <v>46419</v>
+      </c>
+      <c r="H12" s="8" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="13.15">
+      <c r="A13" s="17" t="s">
+        <v>208</v>
+      </c>
+      <c r="B13" s="18">
+        <v>6</v>
+      </c>
+      <c r="C13" s="19">
+        <v>2</v>
+      </c>
+      <c r="D13" s="22">
+        <v>-1</v>
+      </c>
+      <c r="E13" s="22">
+        <v>-10</v>
+      </c>
+      <c r="F13" s="21">
+        <f>IF($I$3="","",EDATE($I$3,B13))</f>
+        <v>46447</v>
+      </c>
+      <c r="H13" s="8" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="13.15">
+      <c r="A14" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="B14" s="16">
+        <v>1</v>
+      </c>
+      <c r="C14" s="11">
+        <v>-0.336146</v>
+      </c>
+      <c r="D14" s="13"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="14">
+        <f>IF($I$3="","",EDATE($I$3,B14))</f>
+        <v>46296</v>
+      </c>
+      <c r="H14" s="8" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="13.15">
+      <c r="A15" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="B15" s="16">
+        <v>2</v>
+      </c>
+      <c r="C15" s="11">
+        <v>-0.67116100000000001</v>
+      </c>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="14">
+        <f>IF($I$3="","",EDATE($I$3,B15))</f>
+        <v>46327</v>
+      </c>
+      <c r="H15" s="8" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="13.15">
+      <c r="A16" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="B16" s="16">
+        <v>3</v>
+      </c>
+      <c r="C16" s="11">
+        <v>-1.0050509999999999</v>
+      </c>
+      <c r="D16" s="13">
+        <v>1</v>
+      </c>
+      <c r="E16" s="13">
+        <v>10</v>
+      </c>
+      <c r="F16" s="14">
+        <f>IF($I$3="","",EDATE($I$3,B16))</f>
+        <v>46357</v>
+      </c>
+      <c r="H16" s="8" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="13.15">
+      <c r="A17" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="B17" s="16">
+        <v>4</v>
+      </c>
+      <c r="C17" s="11">
+        <v>-1.337818</v>
+      </c>
+      <c r="D17" s="13"/>
+      <c r="E17" s="13"/>
+      <c r="F17" s="14">
+        <f>IF($I$3="","",EDATE($I$3,B17))</f>
+        <v>46388</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="13.15">
+      <c r="A18" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="B18" s="16">
+        <v>5</v>
+      </c>
+      <c r="C18" s="11">
+        <v>-1.6694659999999999</v>
+      </c>
+      <c r="D18" s="13"/>
+      <c r="E18" s="13"/>
+      <c r="F18" s="14">
+        <f>IF($I$3="","",EDATE($I$3,B18))</f>
+        <v>46419</v>
+      </c>
+      <c r="H18" s="8" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="13.15">
+      <c r="A19" s="17" t="s">
+        <v>209</v>
+      </c>
+      <c r="B19" s="18">
+        <v>6</v>
+      </c>
+      <c r="C19" s="19">
+        <v>-2</v>
+      </c>
+      <c r="D19" s="22">
+        <v>1</v>
+      </c>
+      <c r="E19" s="22">
+        <v>10</v>
+      </c>
+      <c r="F19" s="21">
+        <f>IF($I$3="","",EDATE($I$3,B19))</f>
+        <v>46447</v>
+      </c>
+      <c r="H19" s="8" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="13.15">
+      <c r="A20" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="B20" s="16">
+        <v>1</v>
+      </c>
+      <c r="C20" s="11">
+        <v>0.81648500000000002</v>
+      </c>
+      <c r="D20" s="13"/>
+      <c r="E20" s="13"/>
+      <c r="F20" s="14">
+        <f>IF($I$3="","",EDATE($I$3,B20))</f>
+        <v>46296</v>
+      </c>
+      <c r="H20" s="8" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="13.15">
+      <c r="A21" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="B21" s="16">
+        <v>2</v>
+      </c>
+      <c r="C21" s="11">
+        <v>1.6396360000000001</v>
+      </c>
+      <c r="D21" s="13"/>
+      <c r="E21" s="13"/>
+      <c r="F21" s="14">
+        <f>IF($I$3="","",EDATE($I$3,B21))</f>
+        <v>46327</v>
+      </c>
+      <c r="H21" s="8" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="13.15">
+      <c r="A22" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="B22" s="16">
+        <v>3</v>
+      </c>
+      <c r="C22" s="11">
+        <v>2.4695079999999998</v>
+      </c>
+      <c r="D22" s="13">
+        <v>-2</v>
+      </c>
+      <c r="E22" s="13">
+        <v>-30</v>
+      </c>
+      <c r="F22" s="14">
+        <f>IF($I$3="","",EDATE($I$3,B22))</f>
+        <v>46357</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="13.15">
+      <c r="A23" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="B23" s="16">
+        <v>4</v>
+      </c>
+      <c r="C23" s="11">
+        <v>3.306155</v>
+      </c>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="14">
+        <f>IF($I$3="","",EDATE($I$3,B23))</f>
+        <v>46388</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="13.15">
+      <c r="A24" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="B24" s="16">
+        <v>5</v>
+      </c>
+      <c r="C24" s="11">
+        <v>4.1496339999999998</v>
+      </c>
+      <c r="D24" s="13"/>
+      <c r="E24" s="13"/>
+      <c r="F24" s="14">
+        <f>IF($I$3="","",EDATE($I$3,B24))</f>
+        <v>46419</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="13.15">
+      <c r="A25" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="B25" s="16">
+        <v>6</v>
+      </c>
+      <c r="C25" s="11">
+        <v>5</v>
+      </c>
+      <c r="D25" s="13">
+        <v>-2</v>
+      </c>
+      <c r="E25" s="13">
+        <v>-30</v>
+      </c>
+      <c r="F25" s="14">
+        <f>IF($I$3="","",EDATE($I$3,B25))</f>
+        <v>46447</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>